<commit_message>
Come here and last save of Fights.csv old fights
</commit_message>
<xml_diff>
--- a/2026-07-11.xlsx
+++ b/2026-07-11.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdsak\OneDrive\Desktop\UFC ML\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74D6DF6C-2D4B-4DEB-92D9-04DDACAF60B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F57041B0-65B4-4788-81F4-C528E7D512B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Predictions" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="82">
   <si>
     <t>Red Corner</t>
   </si>
@@ -70,9 +70,6 @@
     <t>Conor McGregor</t>
   </si>
   <si>
-    <t>+208</t>
-  </si>
-  <si>
     <t>Max Holloway</t>
   </si>
   <si>
@@ -88,15 +85,9 @@
     <t>Benoit Saint Denis</t>
   </si>
   <si>
-    <t>-149</t>
-  </si>
-  <si>
     <t>Paddy Pimblett</t>
   </si>
   <si>
-    <t>+127</t>
-  </si>
-  <si>
     <t>Lightweight</t>
   </si>
   <si>
@@ -106,15 +97,9 @@
     <t>Cory Sandhagen</t>
   </si>
   <si>
-    <t>-152</t>
-  </si>
-  <si>
     <t>Mario Bautista</t>
   </si>
   <si>
-    <t>+130</t>
-  </si>
-  <si>
     <t>Bantamweight</t>
   </si>
   <si>
@@ -124,30 +109,18 @@
     <t>Brandon Royval</t>
   </si>
   <si>
-    <t>+182</t>
-  </si>
-  <si>
     <t>Lone'er Kavanagh</t>
   </si>
   <si>
-    <t>-216</t>
-  </si>
-  <si>
     <t>Flyweight</t>
   </si>
   <si>
     <t>King Green</t>
   </si>
   <si>
-    <t>+132</t>
-  </si>
-  <si>
     <t>Terrance McKinney</t>
   </si>
   <si>
-    <t>-155</t>
-  </si>
-  <si>
     <t>Nikita Krylov</t>
   </si>
   <si>
@@ -157,24 +130,15 @@
     <t>Robert Whittaker</t>
   </si>
   <si>
-    <t>-201</t>
-  </si>
-  <si>
     <t>Light Heavyweight</t>
   </si>
   <si>
     <t>Cody Garbrandt</t>
   </si>
   <si>
-    <t>+321</t>
-  </si>
-  <si>
     <t>Adrian Yanez</t>
   </si>
   <si>
-    <t>-403</t>
-  </si>
-  <si>
     <t>Luke Riley</t>
   </si>
   <si>
@@ -184,66 +148,39 @@
     <t>Kai Kamaka III</t>
   </si>
   <si>
-    <t>+247</t>
-  </si>
-  <si>
     <t>Featherweight</t>
   </si>
   <si>
     <t>Tracy Cortez</t>
   </si>
   <si>
-    <t>+108</t>
-  </si>
-  <si>
     <t>Wang Cong</t>
   </si>
   <si>
-    <t>-126</t>
-  </si>
-  <si>
     <t>Women's Flyweight</t>
   </si>
   <si>
     <t>Damian Pinas</t>
   </si>
   <si>
-    <t>-180</t>
-  </si>
-  <si>
     <t>Cesar Almeida</t>
   </si>
   <si>
-    <t>+153</t>
-  </si>
-  <si>
     <t>Middleweight</t>
   </si>
   <si>
     <t>Ryan Gandra</t>
   </si>
   <si>
-    <t>-166</t>
-  </si>
-  <si>
     <t>Zach Reese</t>
   </si>
   <si>
-    <t>+141</t>
-  </si>
-  <si>
     <t>Cody Durden</t>
   </si>
   <si>
-    <t>+204</t>
-  </si>
-  <si>
     <t>Alessandro Costa</t>
   </si>
   <si>
-    <t>-245</t>
-  </si>
-  <si>
     <t>Predicted Winner</t>
   </si>
   <si>
@@ -272,6 +209,63 @@
   </si>
   <si>
     <t>Blue Odds (Open)</t>
+  </si>
+  <si>
+    <t>No bet</t>
+  </si>
+  <si>
+    <t>+350</t>
+  </si>
+  <si>
+    <t>-500</t>
+  </si>
+  <si>
+    <t>-170</t>
+  </si>
+  <si>
+    <t>+142</t>
+  </si>
+  <si>
+    <t>-200</t>
+  </si>
+  <si>
+    <t>+175</t>
+  </si>
+  <si>
+    <t>-205</t>
+  </si>
+  <si>
+    <t>-116</t>
+  </si>
+  <si>
+    <t>-104</t>
+  </si>
+  <si>
+    <t>+210</t>
+  </si>
+  <si>
+    <t>-400</t>
+  </si>
+  <si>
+    <t>+330</t>
+  </si>
+  <si>
+    <t>+145</t>
+  </si>
+  <si>
+    <t>-265</t>
+  </si>
+  <si>
+    <t>+225</t>
+  </si>
+  <si>
+    <t>+190</t>
+  </si>
+  <si>
+    <t>-225</t>
+  </si>
+  <si>
+    <t>+250</t>
   </si>
 </sst>
 </file>
@@ -311,7 +305,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -333,12 +327,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -586,7 +574,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -658,9 +646,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -673,11 +658,8 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -703,8 +685,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1012,11 +1003,11 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" style="28" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" style="27" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" style="28" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" style="27" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -1026,7 +1017,7 @@
     <col min="13" max="13" width="8" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="6.5703125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="19" max="20" width="17.42578125" bestFit="1" customWidth="1"/>
@@ -1034,45 +1025,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="F1" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="G1" s="35"/>
-      <c r="H1" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="36" t="s">
-        <v>80</v>
-      </c>
-      <c r="P1" s="37"/>
-      <c r="Q1" s="38"/>
-      <c r="R1" s="39" t="s">
-        <v>77</v>
-      </c>
-      <c r="S1" s="40"/>
-      <c r="T1" s="41" t="s">
-        <v>81</v>
-      </c>
-      <c r="U1" s="40"/>
+      <c r="F1" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="33"/>
+      <c r="H1" s="34" t="s">
+        <v>58</v>
+      </c>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="36"/>
+      <c r="R1" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="S1" s="38"/>
+      <c r="T1" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="U1" s="38"/>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="26" t="s">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>2</v>
@@ -1110,19 +1101,19 @@
       <c r="P2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="Q2" s="30" t="s">
+      <c r="Q2" s="29" t="s">
         <v>14</v>
       </c>
       <c r="R2" s="24" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="S2" s="12" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="T2" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="U2" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="U2" s="28" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1130,62 +1121,62 @@
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="42" t="s">
+      <c r="D3" s="31" t="s">
+        <v>65</v>
+      </c>
+      <c r="E3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="8">
+        <v>0.54025945883478288</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="17">
+        <v>0.67733941029981193</v>
+      </c>
+      <c r="J3" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="8">
-        <v>0.54025947900532878</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="I3" s="17">
-        <v>0.61654814170197048</v>
-      </c>
-      <c r="J3" s="23" t="s">
-        <v>20</v>
-      </c>
       <c r="K3" s="3">
-        <v>0.42985203414782852</v>
+        <v>0.42985261859905022</v>
       </c>
       <c r="L3" s="3">
-        <v>0.35319122498009492</v>
+        <v>0.3531915391451606</v>
       </c>
       <c r="M3" s="3">
-        <v>0.42985203414782852</v>
+        <v>0.42985261859905022</v>
       </c>
       <c r="N3" s="17">
-        <v>0.2169567408720767</v>
+        <v>0.21695584225578921</v>
       </c>
       <c r="O3" s="7" t="s">
         <v>15</v>
       </c>
       <c r="P3" s="3">
-        <v>0.38518939532813801</v>
-      </c>
-      <c r="Q3" s="31">
-        <v>4.6296802323093508E-2</v>
+        <v>1.0238157880380709</v>
+      </c>
+      <c r="Q3" s="30">
+        <v>0.1</v>
       </c>
       <c r="R3" s="25" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="S3" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="T3" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="U3" s="16">
         <v>0.62123617940622822</v>
@@ -1193,64 +1184,64 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="42" t="s">
+      <c r="D4" s="31" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="F4" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="8">
+        <v>0.66738754207514428</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="17">
+        <v>0.63616753502764856</v>
+      </c>
+      <c r="J4" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="42" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="8">
-        <v>0.66738754473760264</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" s="17">
-        <v>0.62277255530766662</v>
-      </c>
-      <c r="J4" s="23" t="s">
-        <v>26</v>
-      </c>
       <c r="K4" s="3">
-        <v>0.52836189823760249</v>
+        <v>0.52836043138795208</v>
       </c>
       <c r="L4" s="3">
-        <v>0.2039934119347917</v>
+        <v>0.20399423275448411</v>
       </c>
       <c r="M4" s="3">
-        <v>0.26764468982760581</v>
+        <v>0.26764533585756389</v>
       </c>
       <c r="N4" s="17">
-        <v>0.52836189823760249</v>
-      </c>
-      <c r="O4" s="32" t="s">
-        <v>21</v>
-      </c>
-      <c r="P4" s="27">
-        <v>0.17790014494611461</v>
-      </c>
-      <c r="Q4" s="33">
-        <v>0.05</v>
+        <v>0.52836043138795208</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="P4" s="3">
+        <v>0.11946427171015329</v>
+      </c>
+      <c r="Q4" s="30">
+        <v>0.1</v>
       </c>
       <c r="R4" s="25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="S4" s="13" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="T4" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="U4" s="16">
         <v>0.51204849390065088</v>
@@ -1258,64 +1249,64 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="8">
+        <v>0.51600015088228279</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" s="17">
+        <v>0.58076256177259578</v>
+      </c>
+      <c r="J5" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="42" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="42" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="20" t="s">
+      <c r="K5" s="3">
+        <v>0.45547710258192159</v>
+      </c>
+      <c r="L5" s="3">
+        <v>0.45547710258192159</v>
+      </c>
+      <c r="M5" s="3">
+        <v>0.38844019667566337</v>
+      </c>
+      <c r="N5" s="17">
+        <v>0.1560827007424149</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="P5" s="3">
+        <v>0.29600985880056291</v>
+      </c>
+      <c r="Q5" s="30">
+        <v>8.706172317663613E-2</v>
+      </c>
+      <c r="R5" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="S5" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="8">
-        <v>0.51600014543111228</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I5" s="17">
-        <v>0.54876734446085951</v>
-      </c>
-      <c r="J5" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="K5" s="3">
-        <v>0.45547814708335149</v>
-      </c>
-      <c r="L5" s="3">
-        <v>0.45547814708335149</v>
-      </c>
-      <c r="M5" s="3">
-        <v>0.3884403341491825</v>
-      </c>
-      <c r="N5" s="17">
-        <v>0.15608151876746601</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="P5" s="3">
-        <v>0.10400841390060429</v>
-      </c>
-      <c r="Q5" s="31">
-        <v>2.0001618057808531E-2</v>
-      </c>
-      <c r="R5" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="S5" s="13" t="s">
-        <v>32</v>
-      </c>
       <c r="T5" s="15" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="U5" s="16">
         <v>0.56886441465542059</v>
@@ -1323,64 +1314,64 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="42" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="31" t="s">
         <v>34</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="42" t="s">
-        <v>36</v>
+        <v>29</v>
+      </c>
+      <c r="D6" s="31" t="s">
+        <v>68</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G6" s="8">
-        <v>0.67537457146988467</v>
+        <v>0.67537457035208448</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="I6" s="17">
-        <v>0.66695262589841109</v>
+        <v>0.65930330695534489</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="K6" s="3">
-        <v>0.41379337637306779</v>
+        <v>0.41379342410478559</v>
       </c>
       <c r="L6" s="3">
-        <v>0.41379337637306779</v>
+        <v>0.41379342410478559</v>
       </c>
       <c r="M6" s="3">
-        <v>0.39501099200898121</v>
+        <v>0.3950110199723581</v>
       </c>
       <c r="N6" s="17">
-        <v>0.19119563161795111</v>
-      </c>
-      <c r="O6" s="32" t="s">
-        <v>35</v>
-      </c>
-      <c r="P6" s="27">
-        <v>4.4810391359296098E-2</v>
-      </c>
-      <c r="Q6" s="33">
-        <v>2.4197611334019889E-2</v>
+        <v>0.19119555592285639</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P6" s="3">
+        <v>7.1261285391686968E-2</v>
+      </c>
+      <c r="Q6" s="30">
+        <v>7.1261285391686968E-2</v>
       </c>
       <c r="R6" s="25" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="S6" s="13" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="T6" s="15" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="U6" s="16">
         <v>0.50211081908263977</v>
@@ -1388,64 +1379,64 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="42" t="s">
-        <v>39</v>
+        <v>31</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>69</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" s="42" t="s">
-        <v>41</v>
+        <v>32</v>
+      </c>
+      <c r="D7" s="31" t="s">
+        <v>70</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="G7" s="8">
-        <v>0.52578749567735716</v>
+        <v>0.52578749065827624</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="I7" s="17">
-        <v>0.55563990490693804</v>
+        <v>0.58874273573114899</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="K7" s="3">
-        <v>0.49760349058343067</v>
+        <v>0.49760327630856199</v>
       </c>
       <c r="L7" s="3">
-        <v>0.17274910263910001</v>
+        <v>0.17274898565796259</v>
       </c>
       <c r="M7" s="3">
-        <v>0.32964740677746929</v>
+        <v>0.32964773803347541</v>
       </c>
       <c r="N7" s="17">
-        <v>0.49760349058343067</v>
+        <v>0.49760327630856199</v>
       </c>
       <c r="O7" s="7" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="P7" s="3">
-        <v>8.525355816952751E-2</v>
-      </c>
-      <c r="Q7" s="31">
-        <v>1.6146507229077171E-2</v>
+        <v>0.28639970902305462</v>
+      </c>
+      <c r="Q7" s="30">
+        <v>8.1828488292301299E-2</v>
       </c>
       <c r="R7" s="25" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="S7" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="T7" s="15" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="U7" s="16">
         <v>0.61324359796145311</v>
@@ -1453,64 +1444,60 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B8" s="42" t="s">
-        <v>43</v>
+        <v>33</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>71</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="42" t="s">
-        <v>45</v>
+        <v>35</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>72</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="11">
-        <v>0.51052816934816148</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="I8" s="21">
-        <v>0.56799212985354597</v>
+        <v>36</v>
+      </c>
+      <c r="F8" s="40" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="41">
+        <v>0.51052816628758002</v>
+      </c>
+      <c r="H8" s="42" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="43">
+        <v>0.51176779754859492</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="K8" s="3">
-        <v>0.45115189101094111</v>
+        <v>0.40702628501917643</v>
       </c>
       <c r="L8" s="3">
-        <v>0.38689397067518638</v>
+        <v>0.25512323215791721</v>
       </c>
       <c r="M8" s="3">
-        <v>0.45115189101094111</v>
+        <v>0.33785048282290642</v>
       </c>
       <c r="N8" s="17">
-        <v>0.16195413831387251</v>
+        <v>0.40702628501917643</v>
       </c>
       <c r="O8" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="P8" s="3">
-        <v>0.38552961769747179</v>
-      </c>
-      <c r="Q8" s="31">
-        <v>0.05</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="30"/>
       <c r="R8" s="25" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="S8" s="13" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="T8" s="15" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="U8" s="16">
         <v>0.67195255794776143</v>
@@ -1518,64 +1505,64 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B9" s="42" t="s">
-        <v>48</v>
+        <v>37</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>73</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" s="42" t="s">
-        <v>50</v>
+        <v>38</v>
+      </c>
+      <c r="D9" s="31" t="s">
+        <v>17</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="G9" s="8">
-        <v>0.63323547652149204</v>
+        <v>0.63331913600738843</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="I9" s="17">
-        <v>0.70702229546049478</v>
+        <v>0.66166127618626958</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K9" s="3">
-        <v>0.52147957859669591</v>
+        <v>0.52147960870843735</v>
       </c>
       <c r="L9" s="3">
-        <v>0.32336208131565319</v>
+        <v>0.32336218749618229</v>
       </c>
       <c r="M9" s="3">
-        <v>0.52147957859669591</v>
+        <v>0.52147960870843735</v>
       </c>
       <c r="N9" s="17">
-        <v>0.15515834008765089</v>
+        <v>0.15515820379538051</v>
       </c>
       <c r="O9" s="7" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="P9" s="3">
-        <v>0.41316840756264028</v>
-      </c>
-      <c r="Q9" s="31">
-        <v>3.2178224888056099E-2</v>
+        <v>4.0264055008052413E-2</v>
+      </c>
+      <c r="Q9" s="30">
+        <v>9.5866797638220029E-3</v>
       </c>
       <c r="R9" s="25" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="S9" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="T9" s="15" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="U9" s="16">
         <v>0.50361665972664749</v>
@@ -1583,64 +1570,64 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B10" s="42" t="s">
-        <v>52</v>
+        <v>39</v>
+      </c>
+      <c r="B10" s="31" t="s">
+        <v>74</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D10" s="42" t="s">
-        <v>54</v>
+        <v>41</v>
+      </c>
+      <c r="D10" s="31" t="s">
+        <v>75</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="G10" s="8">
-        <v>0.66636679005983046</v>
+        <v>0.66636678979325825</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="I10" s="17">
-        <v>0.6951134395785129</v>
+        <v>0.72384895304244834</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K10" s="3">
-        <v>0.42778299672786368</v>
+        <v>0.42778296169167801</v>
       </c>
       <c r="L10" s="3">
-        <v>0.37739456843221891</v>
+        <v>0.37739484994420819</v>
       </c>
       <c r="M10" s="3">
-        <v>0.42778299672786368</v>
+        <v>0.42778296169167801</v>
       </c>
       <c r="N10" s="17">
-        <v>0.19482243483991751</v>
+        <v>0.1948221883641138</v>
       </c>
       <c r="O10" s="7" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="P10" s="3">
-        <v>2.832895471435792E-2</v>
-      </c>
-      <c r="Q10" s="31">
-        <v>2.86730310874068E-3</v>
+        <v>0.27429812966429878</v>
+      </c>
+      <c r="Q10" s="30">
+        <v>4.1560322676408912E-2</v>
       </c>
       <c r="R10" s="25" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="S10" s="13" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="T10" s="15" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="U10" s="16">
         <v>0.59190926777854447</v>
@@ -1648,64 +1635,64 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" s="42" t="s">
-        <v>57</v>
+        <v>43</v>
+      </c>
+      <c r="B11" s="31" t="s">
+        <v>66</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="42" t="s">
-        <v>59</v>
+        <v>44</v>
+      </c>
+      <c r="D11" s="31" t="s">
+        <v>76</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="G11" s="8">
-        <v>0.50387527847319169</v>
+        <v>0.50387528332361309</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="I11" s="17">
-        <v>0.52044062945809155</v>
+        <v>0.55205606519828865</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="K11" s="3">
-        <v>0.44290468112829912</v>
+        <v>0.51339938044159916</v>
       </c>
       <c r="L11" s="3">
-        <v>0.44290468112829912</v>
+        <v>0.51339938044159916</v>
       </c>
       <c r="M11" s="3">
-        <v>0.34649345648259883</v>
+        <v>0.24197429542632451</v>
       </c>
       <c r="N11" s="17">
-        <v>0.21060186238910211</v>
+        <v>0.24462632413207619</v>
       </c>
       <c r="O11" s="7" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="P11" s="3">
-        <v>2.9924389455810999E-2</v>
-      </c>
-      <c r="Q11" s="31">
-        <v>6.9269420036599519E-3</v>
+        <v>0.23686792150452129</v>
+      </c>
+      <c r="Q11" s="30">
+        <v>8.1678593622248719E-2</v>
       </c>
       <c r="R11" s="25" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="S11" s="13" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="T11" s="15" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="U11" s="16">
         <v>0.52506393721027933</v>
@@ -1713,64 +1700,64 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" s="42" t="s">
-        <v>62</v>
+        <v>46</v>
+      </c>
+      <c r="B12" s="31" t="s">
+        <v>77</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D12" s="42" t="s">
-        <v>64</v>
+        <v>47</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>78</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="G12" s="8">
-        <v>0.80084794112347546</v>
+        <v>0.80084792918192871</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="I12" s="17">
-        <v>0.71889650589024934</v>
+        <v>0.75492329767872435</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K12" s="3">
-        <v>0.52648828790325719</v>
+        <v>0.52630802041975699</v>
       </c>
       <c r="L12" s="3">
-        <v>0.28142067248909569</v>
+        <v>0.28156185639174042</v>
       </c>
       <c r="M12" s="3">
-        <v>0.52648828790325719</v>
+        <v>0.52630802041975699</v>
       </c>
       <c r="N12" s="17">
-        <v>0.19209103960764709</v>
-      </c>
-      <c r="O12" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="P12" s="27">
-        <v>0.32319278521783817</v>
-      </c>
-      <c r="Q12" s="33">
-        <v>0.05</v>
+        <v>0.19213012318850259</v>
+      </c>
+      <c r="O12" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="P12" s="3">
+        <v>0.1716140805047317</v>
+      </c>
+      <c r="Q12" s="30">
+        <v>0.1</v>
       </c>
       <c r="R12" s="25" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="S12" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="T12" s="15" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="U12" s="16">
         <v>0.51504100667607833</v>
@@ -1778,64 +1765,64 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B13" s="42" t="s">
-        <v>67</v>
+        <v>49</v>
+      </c>
+      <c r="B13" s="31" t="s">
+        <v>79</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="D13" s="42" t="s">
-        <v>69</v>
+        <v>50</v>
+      </c>
+      <c r="D13" s="31" t="s">
+        <v>80</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="F13" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="G13" s="8">
-        <v>0.6440322328776269</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="I13" s="17">
-        <v>0.62257997663720777</v>
+        <v>48</v>
+      </c>
+      <c r="F13" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="G13" s="11">
+        <v>0.64403223132147547</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="I13" s="21">
+        <v>0.51300673650772111</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="K13" s="3">
-        <v>0.56859538211315941</v>
+        <v>0.48018780153418961</v>
       </c>
       <c r="L13" s="3">
-        <v>0.26399379460127531</v>
+        <v>0.2175929069355709</v>
       </c>
       <c r="M13" s="3">
-        <v>0.56859538211315941</v>
+        <v>0.30221929153023952</v>
       </c>
       <c r="N13" s="17">
-        <v>0.16741082328556539</v>
-      </c>
-      <c r="O13" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="P13" s="27">
-        <v>8.5222571362334909E-2</v>
-      </c>
-      <c r="Q13" s="33">
-        <v>3.5367367115368989E-2</v>
+        <v>0.48018780153418961</v>
+      </c>
+      <c r="O13" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="P13" s="3">
+        <v>0.96400806174115661</v>
+      </c>
+      <c r="Q13" s="30">
+        <v>0.1</v>
       </c>
       <c r="R13" s="25" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="S13" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="T13" s="15" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="U13" s="16">
         <v>0.54529260025483939</v>
@@ -1843,64 +1830,64 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B14" s="42" t="s">
-        <v>73</v>
+        <v>52</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>40</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D14" s="42" t="s">
-        <v>71</v>
+        <v>51</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>81</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="G14" s="8">
-        <v>0.58623684978892621</v>
+        <v>0.58623706607369952</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="I14" s="17">
-        <v>0.63622130023747903</v>
+        <v>0.65853128909617853</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K14" s="3">
-        <v>0.4844119375206502</v>
+        <v>0.48441181414722961</v>
       </c>
       <c r="L14" s="3">
-        <v>0.31011280043880463</v>
+        <v>0.31011190970728209</v>
       </c>
       <c r="M14" s="3">
-        <v>0.4844119375206502</v>
+        <v>0.48441181414722961</v>
       </c>
       <c r="N14" s="17">
-        <v>0.2054752620405452</v>
+        <v>0.2054762761454883</v>
       </c>
       <c r="O14" s="7" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="P14" s="3">
-        <v>0.1941264473181219</v>
-      </c>
-      <c r="Q14" s="31">
-        <v>2.3790005798789451E-2</v>
+        <v>0.37481570299449829</v>
+      </c>
+      <c r="Q14" s="30">
+        <v>7.4963140598899664E-2</v>
       </c>
       <c r="R14" s="25" t="s">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="S14" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="T14" s="15" t="s">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="U14" s="16">
         <v>0.6018522695095434</v>

</xml_diff>